<commit_message>
docs(recette): cahier de tests étendu à toutes les fonctionnalités (487 scénarios)
</commit_message>
<xml_diff>
--- a/NEXUSRH_CI_Test_Plan.xlsx
+++ b/NEXUSRH_CI_Test_Plan.xlsx
@@ -791,7 +791,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1000,7 +999,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1472,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2612,7 +2610,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
@@ -2696,34 +2693,12 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:I2"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="C1:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -33261,7 +33236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P64"/>
+  <dimension ref="A1:P69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33285,7 +33260,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MOTEUR DE PAIE CI (CNPS + ITS)  ·  62 scénarios</t>
+          <t xml:space="preserve">  MOTEUR DE PAIE CI (CNPS + ITS)  ·  67 scénarios</t>
         </is>
       </c>
     </row>
@@ -37074,6 +37049,285 @@
         </is>
       </c>
       <c r="P64" s="43" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="58" customHeight="1">
+      <c r="A65" s="51" t="inlineStr">
+        <is>
+          <t>PAY-063</t>
+        </is>
+      </c>
+      <c r="B65" s="44" t="inlineStr">
+        <is>
+          <t>P1 — Critique</t>
+        </is>
+      </c>
+      <c r="C65" s="43" t="inlineStr">
+        <is>
+          <t>Primes soumises CNPS + ITS</t>
+        </is>
+      </c>
+      <c r="D65" s="43" t="inlineStr">
+        <is>
+          <t>Primes d'ancienneté / rendement, heures supp., ICP, gratifications : dans le brut ET dans les bases CNPS et ITS.</t>
+        </is>
+      </c>
+      <c r="E65" s="43" t="inlineStr">
+        <is>
+          <t>Salarié célibataire 200 000 + prime de rendement 50 000</t>
+        </is>
+      </c>
+      <c r="F65" s="43" t="inlineStr">
+        <is>
+          <t>1. Saisir la prime en élément variable
+2. Générer la paie
+3. Ouvrir le bulletin</t>
+        </is>
+      </c>
+      <c r="G65" s="43" t="inlineStr">
+        <is>
+          <t>Brut 250 000 ; CNPS salarié 15 750 (250 000 × 6,3 %) ; base ITS 250 000 ; ITS 28 500 ; net 205 750</t>
+        </is>
+      </c>
+      <c r="H65" s="43" t="n"/>
+      <c r="I65" s="42" t="n"/>
+      <c r="J65" s="43" t="n"/>
+      <c r="K65" s="43" t="n"/>
+      <c r="L65" s="43" t="n"/>
+      <c r="M65" s="43" t="n"/>
+      <c r="N65" s="43" t="n"/>
+      <c r="O65" s="43" t="inlineStr">
+        <is>
+          <t>Recette 10/2026</t>
+        </is>
+      </c>
+      <c r="P65" s="43" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="58" customHeight="1">
+      <c r="A66" s="51" t="inlineStr">
+        <is>
+          <t>PAY-064</t>
+        </is>
+      </c>
+      <c r="B66" s="44" t="inlineStr">
+        <is>
+          <t>P1 — Critique</t>
+        </is>
+      </c>
+      <c r="C66" s="43" t="inlineStr">
+        <is>
+          <t>Prime de transport — plafond d'exonération</t>
+        </is>
+      </c>
+      <c r="D66" s="43" t="inlineStr">
+        <is>
+          <t>Transport exonéré jusqu'à 30 000 F (Abidjan), 24 000 F (Bouaké), 20 000 F (autres villes) ; excédent soumis (CGI art. 116 al. 10 ; arrêté 2020-012/MEPS).</t>
+        </is>
+      </c>
+      <c r="E66" s="43" t="inlineStr">
+        <is>
+          <t>Salarié 200 000 d'une filiale située à Abidjan, prime de transport 45 000</t>
+        </is>
+      </c>
+      <c r="F66" s="43" t="inlineStr">
+        <is>
+          <t>1. Saisir PRIME_TRANSPORT 45 000
+2. Générer la paie
+3. Refaire avec une filiale à Bouaké</t>
+        </is>
+      </c>
+      <c r="G66" s="43" t="inlineStr">
+        <is>
+          <t>Abidjan : base ITS 215 000, CNPS 13 545, ITS 22 400. Bouaké : base 221 000, CNPS 13 923, ITS 23 360. Transport ≤ plafond : aucune incidence sur les bases</t>
+        </is>
+      </c>
+      <c r="H66" s="43" t="n"/>
+      <c r="I66" s="42" t="n"/>
+      <c r="J66" s="43" t="n"/>
+      <c r="K66" s="43" t="n"/>
+      <c r="L66" s="43" t="n"/>
+      <c r="M66" s="43" t="n"/>
+      <c r="N66" s="43" t="n"/>
+      <c r="O66" s="43" t="inlineStr">
+        <is>
+          <t>Recette 10/2026</t>
+        </is>
+      </c>
+      <c r="P66" s="43" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="58" customHeight="1">
+      <c r="A67" s="51" t="inlineStr">
+        <is>
+          <t>PAY-065</t>
+        </is>
+      </c>
+      <c r="B67" s="44" t="inlineStr">
+        <is>
+          <t>P2 — Haute</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>Avantage en nature (ligne 1260 / 5200)</t>
+        </is>
+      </c>
+      <c r="D67" s="43" t="inlineStr">
+        <is>
+          <t>Avantage en nature valorisé au brut, cotisé et imposé, puis repris en retenue (non versé en espèces).</t>
+        </is>
+      </c>
+      <c r="E67" s="43" t="inlineStr">
+        <is>
+          <t>Salarié 200 000 + AVANTAGE_NATURE 50 000 (logement)</t>
+        </is>
+      </c>
+      <c r="F67" s="43" t="inlineStr">
+        <is>
+          <t>1. Saisir l'avantage en élément variable
+2. Générer la paie</t>
+        </is>
+      </c>
+      <c r="G67" s="43" t="inlineStr">
+        <is>
+          <t>Ligne 1260 + 50 000 et ligne 5200 − 50 000 ; CNPS 15 750 ; ITS 28 500 ; net 155 750</t>
+        </is>
+      </c>
+      <c r="H67" s="43" t="n"/>
+      <c r="I67" s="42" t="n"/>
+      <c r="J67" s="43" t="n"/>
+      <c r="K67" s="43" t="n"/>
+      <c r="L67" s="43" t="n"/>
+      <c r="M67" s="43" t="n"/>
+      <c r="N67" s="43" t="n"/>
+      <c r="O67" s="43" t="inlineStr">
+        <is>
+          <t>Recette 10/2026</t>
+        </is>
+      </c>
+      <c r="P67" s="43" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="58" customHeight="1">
+      <c r="A68" s="51" t="inlineStr">
+        <is>
+          <t>PAY-066</t>
+        </is>
+      </c>
+      <c r="B68" s="44" t="inlineStr">
+        <is>
+          <t>P2 — Haute</t>
+        </is>
+      </c>
+      <c r="C68" s="43" t="inlineStr">
+        <is>
+          <t>Assujettissement paramétrable par rubrique</t>
+        </is>
+      </c>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Paramètres → Rubriques de paie : colonnes « Soumis CNPS » / « Imposable ITS » (Selon le pack / Oui / Non).</t>
+        </is>
+      </c>
+      <c r="E68" s="43" t="inlineStr">
+        <is>
+          <t>Rubrique 1200 (VAR:PRIME_RENDEMENT) ; prime 50 000</t>
+        </is>
+      </c>
+      <c r="F68" s="43" t="inlineStr">
+        <is>
+          <t>1. Passer « Imposable ITS » à Non sur la rubrique 1200
+2. Générer la paie
+3. Remettre « Selon le pack »</t>
+        </is>
+      </c>
+      <c r="G68" s="43" t="inlineStr">
+        <is>
+          <t>Étape 2 : CNPS 15 750 (toujours cotisée), base ITS 200 000, ITS 20 000. Étape 3 : retour à base ITS 250 000</t>
+        </is>
+      </c>
+      <c r="H68" s="43" t="n"/>
+      <c r="I68" s="42" t="n"/>
+      <c r="J68" s="43" t="n"/>
+      <c r="K68" s="43" t="n"/>
+      <c r="L68" s="43" t="n"/>
+      <c r="M68" s="43" t="n"/>
+      <c r="N68" s="43" t="n"/>
+      <c r="O68" s="43" t="inlineStr">
+        <is>
+          <t>Recette 10/2026</t>
+        </is>
+      </c>
+      <c r="P68" s="43" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="58" customHeight="1">
+      <c r="A69" s="51" t="inlineStr">
+        <is>
+          <t>PAY-067</t>
+        </is>
+      </c>
+      <c r="B69" s="44" t="inlineStr">
+        <is>
+          <t>P2 — Haute</t>
+        </is>
+      </c>
+      <c r="C69" s="43" t="inlineStr">
+        <is>
+          <t>Congés : acquisition 2,2 j ouvrables / mois</t>
+        </is>
+      </c>
+      <c r="D69" s="43" t="inlineStr">
+        <is>
+          <t>Constante plateforme CONGES_JOURS_PAR_MOIS = 2,2 (CT art. 25.1) ; les bases déjà paramétrées à 2,5 sont migrées sans écraser les autres constantes.</t>
+        </is>
+      </c>
+      <c r="E69" s="43" t="inlineStr">
+        <is>
+          <t>Super-admin : Paramètres plateforme → Constantes légales</t>
+        </is>
+      </c>
+      <c r="F69" s="43" t="inlineStr">
+        <is>
+          <t>1. Ouvrir les constantes légales CI
+2. Vérifier CONGES_JOURS_PAR_MOIS
+3. Vérifier que les autres constantes modifiées sont conservées</t>
+        </is>
+      </c>
+      <c r="G69" s="43" t="inlineStr">
+        <is>
+          <t>CONGES_JOURS_PAR_MOIS = 2,2 ; constantes personnalisées inchangées</t>
+        </is>
+      </c>
+      <c r="H69" s="43" t="n"/>
+      <c r="I69" s="42" t="n"/>
+      <c r="J69" s="43" t="n"/>
+      <c r="K69" s="43" t="n"/>
+      <c r="L69" s="43" t="n"/>
+      <c r="M69" s="43" t="n"/>
+      <c r="N69" s="43" t="n"/>
+      <c r="O69" s="43" t="inlineStr">
+        <is>
+          <t>Recette 10/2026</t>
+        </is>
+      </c>
+      <c r="P69" s="43" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
@@ -37353,13 +37607,13 @@
     <dataValidation sqref="P30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Production,Preprod,Local"</formula1>
     </dataValidation>
-    <dataValidation sqref="I31:I64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I31:I64 I65 I66 I67 I68 I69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✅ Passé,❌ Échoué,⚠️ Bloqué,▶️ En cours,⬜ Non exécuté"</formula1>
     </dataValidation>
-    <dataValidation sqref="B31:B64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"P1 — Critique,P2 — Haute,P3 — Moyenne,P4 — Basse"</formula1>
-    </dataValidation>
-    <dataValidation sqref="P31:P64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B31:B64 B65 B66 B67 B68 B69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"P1 — Critique,P2 — Haute,P3 — Moyenne,P4 — Basse"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P31:P64 P65 P66 P67 P68 P69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Production,Preprod,Local"</formula1>
     </dataValidation>
   </dataValidations>
@@ -37501,7 +37755,7 @@
       </c>
       <c r="D3" s="41" t="inlineStr">
         <is>
-          <t>2.5 jours ouvrables/mois CI</t>
+          <t>2,2 jours ouvrables/mois CI (CT art. 25.1)</t>
         </is>
       </c>
       <c r="E3" s="41" t="inlineStr">

</xml_diff>